<commit_message>
Cập nhật dữ liệu crawl XGEAR 23/10 và gộp các file Excel tổng
</commit_message>
<xml_diff>
--- a/laptop_xgear_all.xlsx
+++ b/laptop_xgear_all.xlsx
@@ -524,12 +524,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T05:09:51+00:00</t>
+          <t>2026-10-21T04:39:25+00:00</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -843,18 +843,18 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Laptop ASUS ProArt P14 H7407BA-SU304W (RTX Spark N1X | RTX Blackwell | 48GB RAM | 1TB SSD | 14 inch 4K OLED 120Hz)</t>
+          <t>Laptop ASUS ProArt P14 H7407BA-SU304W (RTX Spark N1X | RTX Blackwell | 48GB RAM | 1TB SSD | 14 inch 3K OLED 120Hz)</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>114990000</v>
+        <v>113990000</v>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
@@ -866,7 +866,7 @@
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Thương hiệu: Asus | CPU: Nvidia N1x | RAM: 48GB LPDDR5X | VGA: RTX Blackwell | Màn hình: 14" 4K OLED</t>
+          <t>Thương hiệu: Asus | CPU: Nvidia N1x | RAM: 48GB LPDDR5X | VGA: RTX Blackwell | Màn hình: 14" 3K OLED</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T06:42:07+00:00</t>
+          <t>2026-10-22T10:42:41+00:00</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>129990000</v>
+        <v>128990000</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
@@ -952,12 +952,12 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T06:49:10+00:00</t>
+          <t>2026-10-22T10:41:26+00:00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>119990000</v>
+        <v>118990000</v>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
@@ -990,12 +990,12 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T10:10:46+00:00</t>
+          <t>2026-10-22T10:43:08+00:00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>71990000</v>
+        <v>70990000</v>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T05:01:14+00:00</t>
+          <t>2026-10-21T03:28:43+00:00</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>57890000</v>
+        <v>57490000</v>
       </c>
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="inlineStr">
@@ -1258,12 +1258,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T05:07:31+00:00</t>
+          <t>2026-10-21T04:36:59+00:00</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,9 @@
           <t>Laptop ASUS TUF Gaming 16 FX610JP-TU073W (Intel Core 7 14650HX | RTX 5070 | 16GB | 512GB | 16inch 144Hz)</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="n">
+        <v>54990000</v>
+      </c>
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="inlineStr">
         <is>
@@ -1484,12 +1486,12 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T10:12:54+00:00</t>
+          <t>2026-10-20T03:25:20+00:00</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1529,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1560,12 +1562,12 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T05:07:13+00:00</t>
+          <t>2026-10-20T11:21:21+00:00</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1605,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1643,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1681,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1719,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1757,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1795,7 +1797,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1835,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1875,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1915,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1955,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1993,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2033,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2073,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2113,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2153,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2193,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2231,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2269,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2307,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2345,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2385,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2425,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2463,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2503,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2541,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2579,7 +2581,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2621,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2661,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2701,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2741,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2781,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2821,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:44</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2861,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2899,7 +2901,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2941,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2979,7 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3019,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3059,7 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3097,7 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3133,7 +3135,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3175,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3213,7 +3215,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3253,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3291,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3331,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3371,7 @@
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3411,7 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3451,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3491,7 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3529,7 @@
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3567,7 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3603,7 +3605,7 @@
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3645,7 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3683,7 @@
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3723,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3763,7 @@
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3801,7 @@
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3841,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3881,7 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3921,7 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3959,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -3995,7 +3997,7 @@
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4035,7 @@
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4075,7 @@
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4115,7 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4153,7 @@
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4193,7 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4204,7 @@
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>104990000</v>
+        <v>103990000</v>
       </c>
       <c r="C97" s="2" t="inlineStr"/>
       <c r="D97" s="2" t="inlineStr">
@@ -4224,12 +4226,12 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T05:47:13+00:00</t>
+          <t>2026-10-23T02:49:17+00:00</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4269,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4307,7 +4309,7 @@
       </c>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4347,7 @@
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4383,7 +4385,7 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4423,7 @@
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4459,7 +4461,7 @@
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4499,7 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4508,7 +4510,7 @@
         </is>
       </c>
       <c r="B105" s="2" t="n">
-        <v>189990000</v>
+        <v>188990000</v>
       </c>
       <c r="C105" s="2" t="inlineStr"/>
       <c r="D105" s="2" t="inlineStr">
@@ -4530,12 +4532,12 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T04:55:39+00:00</t>
+          <t>2026-10-21T04:49:46+00:00</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4575,7 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4613,7 @@
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4649,7 +4651,7 @@
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4687,7 +4689,7 @@
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4725,7 +4727,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4765,7 +4767,7 @@
       </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4805,7 +4807,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4847,7 @@
       </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4883,7 +4885,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4923,7 @@
       </c>
       <c r="J115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4959,7 +4961,7 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -4997,7 +4999,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5037,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5073,7 +5075,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5113,7 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5149,7 +5151,7 @@
       </c>
       <c r="J121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5187,7 +5189,7 @@
       </c>
       <c r="J122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5225,7 +5227,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5263,7 +5265,7 @@
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5298,12 +5300,12 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T05:34:37+00:00</t>
+          <t>2026-10-22T14:25:19+00:00</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5345,7 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5383,7 +5385,7 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5425,7 @@
       </c>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5463,7 +5465,7 @@
       </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5503,7 +5505,7 @@
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5543,7 +5545,7 @@
       </c>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5583,7 +5585,7 @@
       </c>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5621,7 +5623,7 @@
       </c>
       <c r="J133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5659,7 +5661,7 @@
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5697,7 +5699,7 @@
       </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5735,7 +5737,7 @@
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5773,7 +5775,7 @@
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5813,7 +5815,7 @@
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5853,7 @@
       </c>
       <c r="J139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5889,7 +5891,7 @@
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5927,7 +5929,7 @@
       </c>
       <c r="J141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -5965,7 +5967,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6003,7 +6005,7 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6041,7 +6043,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6077,7 +6079,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6113,7 +6115,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6149,7 +6151,7 @@
       </c>
       <c r="J147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6185,7 +6187,7 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6223,7 +6225,7 @@
       </c>
       <c r="J149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6259,7 +6261,7 @@
       </c>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6297,7 @@
       </c>
       <c r="J151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6337,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6375,7 +6377,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6415,7 +6417,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6455,7 +6457,7 @@
       </c>
       <c r="J155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6493,7 +6495,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6531,7 +6533,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6573,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6611,7 +6613,7 @@
       </c>
       <c r="J159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6622,7 +6624,7 @@
         </is>
       </c>
       <c r="B160" s="2" t="n">
-        <v>61990000</v>
+        <v>61490000</v>
       </c>
       <c r="C160" s="2" t="inlineStr"/>
       <c r="D160" s="2" t="inlineStr">
@@ -6644,12 +6646,12 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T09:31:33+00:00</t>
+          <t>2026-10-23T02:38:36+00:00</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6660,7 +6662,7 @@
         </is>
       </c>
       <c r="B161" s="2" t="n">
-        <v>61990000</v>
+        <v>61490000</v>
       </c>
       <c r="C161" s="2" t="inlineStr"/>
       <c r="D161" s="2" t="inlineStr">
@@ -6682,12 +6684,12 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T09:20:43+00:00</t>
+          <t>2026-10-23T02:39:28+00:00</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6725,7 +6727,7 @@
       </c>
       <c r="J162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6765,7 +6767,7 @@
       </c>
       <c r="J163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6805,7 +6807,7 @@
       </c>
       <c r="J164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6843,7 +6845,7 @@
       </c>
       <c r="J165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6881,7 +6883,7 @@
       </c>
       <c r="J166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6923,7 @@
       </c>
       <c r="J167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -6961,7 +6963,7 @@
       </c>
       <c r="J168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7001,7 +7003,7 @@
       </c>
       <c r="J169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7041,7 +7043,7 @@
       </c>
       <c r="J170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7083,7 @@
       </c>
       <c r="J171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7121,7 +7123,7 @@
       </c>
       <c r="J172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7161,7 +7163,7 @@
       </c>
       <c r="J173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7201,7 +7203,7 @@
       </c>
       <c r="J174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7241,7 +7243,7 @@
       </c>
       <c r="J175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7279,7 +7281,7 @@
       </c>
       <c r="J176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7321,7 @@
       </c>
       <c r="J177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7354,12 +7356,12 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T15:19:41+00:00</t>
+          <t>2026-10-23T02:18:38+00:00</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7399,7 +7401,7 @@
       </c>
       <c r="J179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7441,7 @@
       </c>
       <c r="J180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7481,7 @@
       </c>
       <c r="J181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:48</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7517,7 +7519,7 @@
       </c>
       <c r="J182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7557,7 +7559,7 @@
       </c>
       <c r="J183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7595,7 +7597,7 @@
       </c>
       <c r="J184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7633,7 +7635,7 @@
       </c>
       <c r="J185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7673,7 +7675,7 @@
       </c>
       <c r="J186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7713,7 +7715,7 @@
       </c>
       <c r="J187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7751,7 +7753,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7789,7 +7791,7 @@
       </c>
       <c r="J189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7831,7 @@
       </c>
       <c r="J190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7867,7 +7869,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7907,7 +7909,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7947,7 +7949,7 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -7985,7 +7987,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8023,7 +8025,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8061,7 +8063,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8101,7 +8103,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8143,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8181,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8221,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8257,7 +8259,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8268,7 +8270,7 @@
         </is>
       </c>
       <c r="B202" s="2" t="n">
-        <v>33990000</v>
+        <v>32990000</v>
       </c>
       <c r="C202" s="2" t="inlineStr"/>
       <c r="D202" s="2" t="inlineStr">
@@ -8290,12 +8292,12 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T04:35:56+00:00</t>
+          <t>2026-10-23T02:33:12+00:00</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8306,7 +8308,7 @@
         </is>
       </c>
       <c r="B203" s="2" t="n">
-        <v>28990000</v>
+        <v>27490000</v>
       </c>
       <c r="C203" s="2" t="inlineStr"/>
       <c r="D203" s="2" t="inlineStr">
@@ -8328,12 +8330,12 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T03:48:51+00:00</t>
+          <t>2026-10-23T02:33:56+00:00</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8373,7 +8375,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8411,7 +8413,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8422,7 +8424,7 @@
         </is>
       </c>
       <c r="B206" s="2" t="n">
-        <v>32690000</v>
+        <v>31590000</v>
       </c>
       <c r="C206" s="2" t="inlineStr"/>
       <c r="D206" s="2" t="inlineStr">
@@ -8444,12 +8446,12 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T03:49:47+00:00</t>
+          <t>2026-10-23T02:29:07+00:00</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8489,7 +8491,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8527,7 +8529,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8565,7 +8567,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8603,7 +8605,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8641,7 +8643,7 @@
       </c>
       <c r="J211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8679,7 +8681,7 @@
       </c>
       <c r="J212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8717,7 +8719,7 @@
       </c>
       <c r="J213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8757,7 @@
       </c>
       <c r="J214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8793,7 +8795,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8831,7 +8833,7 @@
       </c>
       <c r="J216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8869,7 +8871,7 @@
       </c>
       <c r="J217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8907,7 +8909,7 @@
       </c>
       <c r="J218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8945,7 +8947,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -8985,7 +8987,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9023,7 +9025,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9063,7 +9065,7 @@
       </c>
       <c r="J222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9096,12 +9098,12 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T07:11:21+00:00</t>
+          <t>2026-10-22T15:21:42+00:00</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9134,12 +9136,12 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T07:11:04+00:00</t>
+          <t>2026-10-22T15:19:36+00:00</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9177,7 +9179,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9215,7 +9217,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9255,7 +9257,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9295,7 +9297,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9337,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9370,12 +9372,12 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T07:32:04+00:00</t>
+          <t>2026-10-22T15:27:31+00:00</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9415,7 +9417,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9455,7 +9457,7 @@
       </c>
       <c r="J232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9495,7 +9497,7 @@
       </c>
       <c r="J233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9533,7 +9535,7 @@
       </c>
       <c r="J234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9571,7 +9573,7 @@
       </c>
       <c r="J235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9609,7 +9611,7 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9649,7 @@
       </c>
       <c r="J237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9685,7 +9687,7 @@
       </c>
       <c r="J238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9696,7 +9698,7 @@
         </is>
       </c>
       <c r="B239" s="2" t="n">
-        <v>139990000</v>
+        <v>142990000</v>
       </c>
       <c r="C239" s="2" t="inlineStr"/>
       <c r="D239" s="2" t="inlineStr">
@@ -9718,12 +9720,12 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T07:13:51+00:00</t>
+          <t>2026-10-20T04:49:17+00:00</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9761,7 +9763,7 @@
       </c>
       <c r="J240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9799,7 +9801,7 @@
       </c>
       <c r="J241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:55:30</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9837,7 +9839,7 @@
       </c>
       <c r="J242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9875,7 +9877,7 @@
       </c>
       <c r="J243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9915,7 +9917,7 @@
       </c>
       <c r="J244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9955,7 +9957,7 @@
       </c>
       <c r="J245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -9995,7 +9997,7 @@
       </c>
       <c r="J246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10030,12 +10032,12 @@
       </c>
       <c r="I247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T07:33:51+00:00</t>
+          <t>2026-10-20T02:33:47+00:00</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10075,7 +10077,7 @@
       </c>
       <c r="J248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10113,7 +10115,7 @@
       </c>
       <c r="J249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10153,7 +10155,7 @@
       </c>
       <c r="J250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10193,7 +10195,7 @@
       </c>
       <c r="J251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10233,7 +10235,7 @@
       </c>
       <c r="J252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10271,7 +10273,7 @@
       </c>
       <c r="J253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10309,7 +10311,7 @@
       </c>
       <c r="J254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10349,7 +10351,7 @@
       </c>
       <c r="J255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10387,7 +10389,7 @@
       </c>
       <c r="J256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10427,7 +10429,7 @@
       </c>
       <c r="J257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10467,7 +10469,7 @@
       </c>
       <c r="J258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10507,7 +10509,7 @@
       </c>
       <c r="J259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10547,7 +10549,7 @@
       </c>
       <c r="J260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10587,7 @@
       </c>
       <c r="J261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10623,7 +10625,7 @@
       </c>
       <c r="J262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10661,7 +10663,7 @@
       </c>
       <c r="J263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10697,7 +10699,7 @@
       </c>
       <c r="J264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10737,7 +10739,7 @@
       </c>
       <c r="J265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10775,7 +10777,7 @@
       </c>
       <c r="J266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10813,7 +10815,7 @@
       </c>
       <c r="J267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10851,7 +10853,7 @@
       </c>
       <c r="J268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10889,7 +10891,7 @@
       </c>
       <c r="J269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10925,7 +10927,7 @@
       </c>
       <c r="J270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -10963,7 +10965,7 @@
       </c>
       <c r="J271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11003,7 +11005,7 @@
       </c>
       <c r="J272" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11041,7 +11043,7 @@
       </c>
       <c r="J273" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11079,7 +11081,7 @@
       </c>
       <c r="J274" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11117,7 +11119,7 @@
       </c>
       <c r="J275" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11157,7 +11159,7 @@
       </c>
       <c r="J276" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11197,7 +11199,7 @@
       </c>
       <c r="J277" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11235,7 +11237,7 @@
       </c>
       <c r="J278" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11273,7 +11275,7 @@
       </c>
       <c r="J279" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11313,7 +11315,7 @@
       </c>
       <c r="J280" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11353,7 +11355,7 @@
       </c>
       <c r="J281" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11391,7 +11393,7 @@
       </c>
       <c r="J282" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11429,7 +11431,7 @@
       </c>
       <c r="J283" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11467,7 +11469,7 @@
       </c>
       <c r="J284" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11500,12 +11502,12 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T07:29:27+00:00</t>
+          <t>2026-10-20T04:21:30+00:00</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11538,12 +11540,12 @@
       </c>
       <c r="I286" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T07:29:18+00:00</t>
+          <t>2026-10-20T04:22:20+00:00</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11581,7 +11583,7 @@
       </c>
       <c r="J287" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11621,7 +11623,7 @@
       </c>
       <c r="J288" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11635,11 +11637,11 @@
         <v>32990000</v>
       </c>
       <c r="C289" s="2" t="n">
-        <v>37990000</v>
+        <v>38990000</v>
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>-13%</t>
+          <t>-15%</t>
         </is>
       </c>
       <c r="E289" s="2" t="inlineStr"/>
@@ -11656,12 +11658,12 @@
       </c>
       <c r="I289" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T09:11:13+00:00</t>
+          <t>2026-10-22T07:20:17+00:00</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11699,7 +11701,7 @@
       </c>
       <c r="J290" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11737,7 +11739,7 @@
       </c>
       <c r="J291" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11775,7 +11777,7 @@
       </c>
       <c r="J292" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11813,7 +11815,7 @@
       </c>
       <c r="J293" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11851,7 +11853,7 @@
       </c>
       <c r="J294" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11862,7 +11864,7 @@
         </is>
       </c>
       <c r="B295" s="2" t="n">
-        <v>20890000</v>
+        <v>21890000</v>
       </c>
       <c r="C295" s="2" t="inlineStr"/>
       <c r="D295" s="2" t="inlineStr">
@@ -11884,12 +11886,12 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T12:18:18+00:00</t>
+          <t>2026-10-20T11:45:35+00:00</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11900,7 +11902,7 @@
         </is>
       </c>
       <c r="B296" s="2" t="n">
-        <v>118690000</v>
+        <v>116890000</v>
       </c>
       <c r="C296" s="2" t="inlineStr"/>
       <c r="D296" s="2" t="inlineStr">
@@ -11922,12 +11924,12 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>2026-06-26T12:42:59+00:00</t>
+          <t>2026-10-20T11:57:28+00:00</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -11965,7 +11967,7 @@
       </c>
       <c r="J297" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -12003,7 +12005,7 @@
       </c>
       <c r="J298" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>
@@ -12041,7 +12043,7 @@
       </c>
       <c r="J299" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 07:56:12</t>
+          <t>2026-10-23 09:55:18</t>
         </is>
       </c>
     </row>

</xml_diff>